<commit_message>
add agriculture datasets to site
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W36"/>
+  <dimension ref="A1:W44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3646,25 +3646,97 @@
       <c r="W35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ui_35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Eyes on the Ground Image Data</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Smallholder Farmer Field Monitoring with Machine Learning</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>This machine learning dataset of smallholder farmer's fields includes georeferenced crop images along with labels on input use, crop management, phenology, crop damage, and yields, collected across 8 counties in Kenya. This dataset enables the development of AI systems to monitor crop conditions, predict yields, and support agricultural decision-making for smallholder farmers.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://radiantearth.github.io/stac-browser/#/external/raw.githubusercontent.com/khufkens/EotG_data/main/release_v1/EotG_images/catalog.json</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Images, Geospatial/Remote Sensing</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Lilian Waithaka, Koen Hufkens, Berber Kramer and Benson Njuguna</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Georeferenced crop images with labels on input use, crop management, phenology, crop damage, and yields from 8 counties in Kenya. Machine learning ready dataset for smallholder agriculture monitoring.</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Enables crop monitoring, yield prediction, and agricultural decision support systems for smallholder farmers.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>This dataset can be used to develop AI applications for crop monitoring, yield estimation, damage assessment, and agricultural advisory services. It supports the development of precision agriculture tools specifically designed for smallholder farming systems.</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Authors: Lilian Waithaka, Koen Hufkens, Berber Kramer and Benson Njuguna</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Lilian Waithaka, Koen Hufkens, Berber Kramer and Benson Njuguna</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Computer Vision, Remote Sensing</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr">
         <is>
@@ -3673,6 +3745,826 @@
       </c>
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ui_36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>High-Accuracy Maize Plot Location and Yield Dataset in East Africa</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Corrected Geolocations for Eastern Africa Crop Cut Yield Estimation</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>This dataset includes corrected geolocations of fields, improving the usability of the most expansive Eastern Africa crop cut yield estimation. Collected by the non-profit One Acre Fund from 2015 – 2019, this dataset covers major crop producing regions in Kenya, Rwanda, and Tanzania. It enables accurate yield mapping and agricultural monitoring across East Africa.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/140eLeY3Z_JALFa0B77ZTP9gFt-mSPWXl</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Tabular, Geospatial/Remote Sensing</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>One Acre Fund</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Kenya, Rwanda, Tanzania</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Corrected geolocations of maize fields with yield data from 2015-2019 covering major crop producing regions in Kenya, Rwanda, and Tanzania. Most expansive Eastern Africa crop cut yield estimation dataset.</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Enables accurate yield mapping, crop monitoring, and agricultural planning across East Africa using corrected geolocation data.</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>This dataset can be used for yield prediction modeling, agricultural policy planning, food security assessments, and developing precision agriculture applications for East African smallholder farmers.</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>One Acre Fund</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>One Acre Fund</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Agricultural Informatics, Geospatial Analysis</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ui_37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sensor Based Aquaponics Fish Pond Datasets: IoT Fish Pond Monitoring Datasets</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>IoT Water Quality Management for Aquaponics Systems</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>This project built a remotely monitored and controlled Internet of Things (IoT) fish pond water quality management system for the generation of labeled datasets both for conventional ponds and the aquaponic pond systems. It enables monitoring and optimization of water quality parameters for sustainable aquaculture.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.kaggle.com/ogbuokiriblessing/sensor-based-aquaponics-fish-pond-datasets</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture), SDG 6 (Clean water and sanitation)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Tabular, IoT Sensor Data</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Udanor Collins, Blessing Ogbuokiri, and Nweke Onyiny</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>IoT sensor data from fish pond water quality monitoring systems including conventional ponds and aquaponic systems. Labeled datasets for water quality parameters monitoring.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Enables automated water quality monitoring, predictive maintenance for aquaculture systems, and optimization of aquaponics operations.</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>This dataset can be used to develop IoT-based monitoring systems for aquaculture, predictive models for water quality management, and automated control systems for sustainable fish farming operations.</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Authors: Udanor Collins, Blessing Ogbuokiri, and Nweke Onyiny</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Udanor Collins, Blessing Ogbuokiri, and Nweke Onyiny</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>IoT, Aquaculture Technology</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ui_38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Machine Learning Datasets for Crop Pest and Disease Diagnosis: Crop Imagery and Spectrometry Data</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>AI-Powered Crop Disease Detection for Food Security Crops</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>This dataset contains a repository of image and spectrometry datasets for five main food security crops in Sub-Saharan Africa: cassava, maize, beans, bananas, and cocoa. Collected and curated in collaboration with the in-country agricultural experts, the datasets deliver a wide range of machine learning applications, including classification, object detection, early crop disease detection, and spatial analysis. The team collected and annotated 127,046 images and 39,300 spectral data points.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://dataverse.harvard.edu/dataverse/airlabug/</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Images, Spectrometry Data</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Joyce Nakatumba-Nabende, Andrew Katumba, Claire Babirye, Jeremy Francis Tusubira, Godliver Owomugisha, Neema Mduma, Darlington Akogo, Blessing Sibanda</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Uganda, Tanzania, Ghana</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>127,046 images and 39,300 spectral data points for cassava, maize, beans, bananas, and cocoa. Annotated datasets for classification, object detection, early crop disease detection, and spatial analysis.</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Enables crop disease classification, early detection systems, pest identification, and spatial analysis for food security crops in Sub-Saharan Africa.</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>This dataset can be used to develop mobile applications for crop disease diagnosis, early warning systems for pest outbreaks, and precision agriculture tools for smallholder farmers growing food security crops.</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Authors: Joyce Nakatumba-Nabende, Andrew Katumba, Claire Babirye, Jeremy Francis Tusubira, Godliver Owomugisha, Neema Mduma, Darlington Akogo, Blessing Sibanda</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Joyce Nakatumba-Nabende, Andrew Katumba, Claire Babirye, Jeremy Francis Tusubira, Godliver Owomugisha, Neema Mduma, Darlington Akogo, Blessing Sibanda</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Computer Vision, Agricultural Technology</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ui_39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>A Decision-Supporting Tool for Developing Community-led Land Use Plans</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Pastoral Community Land Use and Livestock Movement Patterns</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>This dataset focuses on locations with predominantly pastoral communities in northern Tanzania to identify fine and broad-scale movements of livestock and land use patterns and to understand how these relate to communal conflicts. It is a high-quality, accurate and labeled dataset containing detailed information on ~ 2000 communal resources (e.g., rangelands, water points, and dips) and their use patterns for over 220 villages across four large districts in northern Tanzania, representative of pastoral systems of livestock production in East Africa.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>http://dtlp.nottech.co.tz/index.html</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture), SDG 16 (Peace, Justice and Strong Institutions)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Geospatial/Remote Sensing, Tabular</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Gladness Mwanga (gladnessg@nm-aist.ac.tz), Divine Ekwem (divine.ekwem@glasgow.ac.uk)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Detailed information on ~2000 communal resources and use patterns for over 220 villages across four districts in northern Tanzania. Covers rangelands, water points, dips and livestock movement patterns.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Enables land use planning, conflict prediction, livestock migration route identification, and infrastructure placement for pastoral communities.</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>This dataset can be used to develop tools for community land use planning, conflict early warning systems, infrastructure development planning for pastoral areas, and sustainable rangeland management systems.</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Authors: Dr. Divine Ekwem (University of Glasgow), Gladness Mwanga (Nelson Mandela African Institution of Science and Technology), Professor Gabriel Shirima (Nelson Mandela African Institution of Science and Technology), Professor Mizech Chagunda (University of Hohenheim)</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Dr. Divine Ekwem, Gladness Mwanga, Professor Gabriel Shirima, Professor Mizech Chagunda</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Geospatial Analysis, Land Use Planning</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ui_40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Enhanced Agriculture Datasets for Remote Crop Monitoring to Provide Access to Essential Social and Financial Services to Smallholder Farmers in Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Yield Prediction and Crop Insurance for Smallholder Farmers</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>The project created labeled yield estimates from 3000 farmers, and was used to train prediction models for yield prediction across the country, consequently using the dataset to generate high resolution crop mask layers for the different value chains. The yield prediction models were enhanced by other biophysical datasets ranging from soil properties and climate related indicators. The datasets proved a concept of scalable machine learning models training, which may be able to respond more appropriately and cost-effectively to agricultural stressors.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://zenodo.org/records/10060610</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture), SDG 1 (No Poverty)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Tabular, Geospatial/Remote Sensing</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Seth Odhiambo (sodhiambo@pula.io)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Labeled yield estimates from 3000 farmers with biophysical datasets including soil properties and climate indicators. High resolution crop mask layers for different value chains.</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Enables yield prediction models, crop insurance products, and agricultural risk assessment for smallholder farmers accessing financial services.</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>This dataset can be used to develop crop insurance products, yield prediction systems, agricultural lending platforms, and risk assessment tools for financial institutions serving smallholder farmers.</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Pula Advisors</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Seth Odhiambo, Pula Advisors</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Dataset &gt; Model</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Agricultural Technology, Financial Technology</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ui_41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>A region-wide, multi-year set of crop field boundary labels for Africa</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Continental Crop Field Boundary Detection</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>This dataset provides continent-wide crop field labels for Africa, improving the availability and use of crop field boundary (parcel) maps. It contains 42,403 annotated geospatial polygons indicating the boundaries of individual crop fields spanning the years 2017-2023. This enables the development of automated field boundary detection systems for agricultural monitoring across Africa.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://zenodo.org/records/11060871</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://github.com/agroimpacts/lacunalabels</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Geospatial/Remote Sensing</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Mary Dziedzorm Afenyo (mary@farmerline.co), Lyndon Estes (lestes@clarku.edu), Primož Kovačič (primoz@spatialcollective.com)</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Multi-country Africa</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>42,403 annotated geospatial polygons of crop field boundaries spanning 2017-2023 across Africa. Continent-wide dataset for field boundary detection.</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Enables automated crop field boundary detection, agricultural area estimation, and crop monitoring systems across Africa.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>This dataset can be used to develop automated field boundary detection systems, agricultural statistics generation, crop area estimation tools, and satellite-based monitoring systems for African agriculture.</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Farmerline, Clark University, Spatial Collective</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Wussah, A., Afenyo, M., Osei, A.K., Gathigi, M., Kovačič, P., Muhando, J., Addai, F., Akakpo, E.S., Allotey, M., Amkoya, P., Amponsem, E., Dadon, K.D., Gyan, V., Harrison X.G., Heltzel, E., Juma, C., Mdawida, R., Miroyo, A., Mucha, J., Mugami, J., Mwawaza, F., Nyarko, D., Oduor, P., Ohemeng, K., Segbefia, S.I.D., Tumbula, T., Wambua, F., Yeboah, F., Estes, L.D.</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Computer Vision, Remote Sensing</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>GitHub: https://github.com/agroimpacts/lacunalabels, AWS Open Data Registry: https://registry.opendata.aws/africa-field-boundary-labels/</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ui_42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CropHarvest: Informing decision-making around agricultural development, early warning systems, and trade in Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Crop Type Classification for Agricultural Decision Making</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CropHarvest increases the understanding of the main types of food production in Sub-Saharan Africa and can help inform decision-making around agricultural development, early warning systems, and regional trade. It is a global, open-source remote sensing dataset for crop-type classification in Sub-Saharan Africa – specifically in Kenya, Mali, Togo, Rwanda, Uganda, Ethiopia, Malawi, Zambia, Tanzania, Namibia, Sudan, and Nigeria. The team expanded on an existing dataset to include new labeled data points, ground data for crop type mapping, street-level images, crowdsourced labeled images, and price data.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://github.com/nasaharvest/cropharvest</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Geospatial/Remote Sensing, Images</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Catherine Nakalembe (cnakalem@umd.edu)</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Kenya, Mali, Togo, Rwanda, Uganda, Ethiopia, Malawi, Zambia, Tanzania, Namibia, Sudan, Nigeria</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Remote sensing dataset for crop-type classification across 12 Sub-Saharan African countries. Includes labeled data points, ground data, street-level images, and price data.</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Enables crop type classification, agricultural development planning, early warning systems, and regional trade analysis for Sub-Saharan Africa.</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>This dataset can be used to develop crop monitoring systems, early warning systems for food security, agricultural trade analysis tools, and policy support systems for agricultural development.</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>NASA Harvest, University of Maryland</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Tseng, G., Zvonkov, I., Nakalembe, C.L., Kerner, H.</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Dataset &gt; Model</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Remote Sensing, Agricultural Informatics</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>https://zenodo.org/record/7257688#.ZFATwuzMI0Q</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ui_43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Improving livelihoods in Ghana and Uganda: Drone-based Agricultural Dataset for Crop Yield Estimation of cashew, cocoa, and coffee</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Drone-Based Crop Yield Estimation for Tree Crops</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>This dataset supports yield estimation, crop type detection and classification, fruit detection and counting, and fruit maturity stage detection (unripe, ripe, and spoiled) for three products that are important sources of livelihood for millions of households in Sub-Saharan Africa. It contains 14,870 drone images with bounding box annotations of cashew, cocoa, and coffee trees collected across multiple farms in Ghana and Uganda. This dataset will help transform African agriculture into agribusiness by allowing for the development of yield estimation solutions that enable farmers to make good business decisions.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/datasets/KaraAgroAI/Drone-based-Agricultural-Dataset-for-Crop-Yield-Estimation</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>SDG 2 (End hunger, achieve food security, sustainable agriculture), SDG 1 (No Poverty)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Images, Drone Imagery</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Darlington Akogo (darlington@gudra-studio.com)</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Ghana, Uganda</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>14,870 drone images with bounding box annotations of cashew, cocoa, and coffee trees. Supports yield estimation, crop type detection, fruit detection and counting, and maturity stage detection.</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Enables automated yield estimation, harvest planning, fruit quality assessment, and business decision support for tree crop farmers.</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>This dataset can be used to develop mobile applications for yield estimation, harvest timing optimization tools, fruit quality assessment systems, and agricultural business planning platforms for tree crop farmers.</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>KaraAgro AI, Makerere AI Lab</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Darlington Akogo, Cyril Akafia, Harriet Fiagbor, Stephen Torkpo, Christian Kusi, Joyce Nakatumba-Nabende</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Computer Vision, Drone Technology</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>agriculture-banner.jpg</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add language dataset docs
</commit_message>
<xml_diff>
--- a/docs/data_catalog.xlsx
+++ b/docs/data_catalog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X55"/>
+  <dimension ref="A1:X72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5666,6 +5666,1502 @@
       </c>
       <c r="X55" t="inlineStr"/>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ui_55</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>A Nigerian Twitter Sentiment Corpus for Multilingual Sentiment Analysis</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>This dataset is the first large-scale human-annotated Twitter sentiment dataset for Hausa, Igbo, Nigerian-Pidgin, and Yorùbá, the four most widely spoken languages in Nigeria.</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://github.com/hausanlp/NaijaSenti</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Shamsuddeen Hassan Muhammad, David Ifeoluwa Adelani, Sebastian Ruder, Ibrahim Said Ahmad, Idris Abdulmumin, Bello Shehu Bello, Monojit Choudhury, Chris Chinenye Emezue, Saheed Salahudeen Abdullahi, Anuoluwapo Aremu, Alipio Jeorge, and Pavel Brazdil</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Powered by: Multiple authors collaboration
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Shamsuddeen Hassan Muhammad, David Ifeoluwa Adelani, Sebastian Ruder, Ibrahim Said Ahmad, Idris Abdulmumin, Bello Shehu Bello, Monojit Choudhury, Chris Chinenye Emezue, Saheed Salahudeen Abdullahi, Anuoluwapo Aremu, Alipio Jeorge, Pavel Brazdil (Multiple authors collaboration)</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ui_56</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Machine Translation Benchmark Dataset for Languages in the Horn of Africa</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>This evaluation dataset automatically quantifies the quality of machine translation systems for Afar, Amharic, Oromo, Somali and Tigrinya.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://github.com/asmelashteka/HornMT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Asmelash Teka Hadgu, Gebrekirstos G. Gebremeskel, Abel Aregawi</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Horn of Africa (Ethiopia, Eritrea)</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Powered by: Horn of Africa research collaboration
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Asmelash Teka Hadgu, Gebrekirstos G. Gebremeskel, Abel Aregawi (Horn of Africa research collaboration)</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr"/>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr"/>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ui_57</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Kencorpus: Kenyan Languages Corpus for Machine Learning and Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>This project collected text and speech corpora for three languages in Kenya: Kiswahili, Dholuo and 3 Luhya dialects (Lumarachi, Logooli and Lubukusu). A total of 4,442 texts were collected and 1,152 files containing spontaneous speech data totaling 176 hours.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.7910/DVN/6N5V1K</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Owen McOnyango (Maseno University), Florence Indede (Maseno University), Lilian D.A. Wanzare (Maseno University), Barack Wanjawa (University of Nairobi), Edward Ombui (Africa Nazarene University), Lawrence Muchemi (University of Nairobi)</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Powered by: Maseno University, University of Nairobi, Africa Nazarene University
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Owen McOnyango, Florence Indede, Lilian D.A. Wanzare (Maseno University), Barack Wanjawa, Lawrence Muchemi (University of Nairobi), Edward Ombui (Africa Nazarene University)</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr"/>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ui_58</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>KenPos: Kenyan Languages Part of Speech Tagged dataset</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>This project developed a Part of Speech (POS) Tagged dataset of 2 languages in Kenya: Dholuo and 3 Luhya dialects (Lumarachi, Lulogooli, and Lubukusi). The project tagged approximately 143,000 words.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.7910/DVN/KLCKL5</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Florence Indede (Maseno University), Owen McOnyango (Maseno University), Lilian D.A. Wanzare (Maseno University), Barack Wanjawa (University of Nairobi), Edward Ombui (Africa Nazarene University), Lawrence Muchemi (University of Nairobi)</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Powered by: Maseno University, University of Nairobi, Africa Nazarene University
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Florence Indede, Owen McOnyango, Lilian D.A. Wanzare (Maseno University), Barack Wanjawa, Lawrence Muchemi (University of Nairobi), Edward Ombui (Africa Nazarene University)</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr"/>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ui_59</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>KenSpeech: Swahili Speech Transcriptions</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>This project produced a speech dataset that includes both read and spontaneous speech recordings, recorded in Kenya with native Swahili speakers, and corresponding transcripts. In total, the dataset includes 27 hours, 31 minutes, 50 seconds of speech data from 26 speakers.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.7910/DVN/YHXJSU</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Dorcas Awino (University of Nairobi), Lawrence Muchemi (University of Nairobi), Lilian D.A. Wanzare (Maseno University), Edward Ombui (Africa Nazarene University), Barack Wanjawa (Maseno University), Owen McOnyango (Maseno University), Florence Indede (Maseno University)</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Powered by: University of Nairobi, Maseno University, Africa Nazarene University
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Dorcas Awino, Lawrence Muchemi (University of Nairobi), Lilian D.A. Wanzare, Barack Wanjawa, Owen McOnyango, Florence Indede (Maseno University), Edward Ombui (Africa Nazarene University)</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr"/>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ui_60</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>KenTrans: A Parallel Corpora for Swahili and local Kenyan Languages</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>This project produced a parallel corpus between Swahili and two other Kenya Languages: Dholuo and 3 Luhya dialects (Lumarachi, Logooli and Lubukusu). A total of about 12,400 sentences were translated to Kiswahili.</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.7910/DVN/NOAT0W</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Lilian D.A Wanzare (Maseno University), Florence Indede (Maseno University), Owen McOnyango (Maseno University), Edward Ombui (Africa Nazarene University), Barack Wanjawa (University of Nairobi), Lawrence Muchemi (University of Nairobi)</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Powered by: Maseno University, University of Nairobi, Africa Nazarene University
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Lilian D.A Wanzare, Florence Indede, Owen McOnyango (Maseno University), Barack Wanjawa, Lawrence Muchemi (University of Nairobi), Edward Ombui (Africa Nazarene University)</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ui_61</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>KenSwQuAD – A Question Answering Dataset for Swahili Low Resource Language</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>This project produced a large Machine Reading Comprehension dataset for the Kiswahili Language. A total of 7,526 Question-Answer (QA) pairs were developed based on 1,445 Swahili story texts.</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.7910/DVN/OTL0LM</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Barack Wanjawa (University of Nairobi), Lilian D.A. Wanzare (Maseno University), Florence Indede (Maseno University), Owen McOnyango (Maseno University), Lawrence Muchemi (University of Nairobi), Edward Ombui (Africa Nazarene University)</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Powered by: University of Nairobi, Maseno University, Africa Nazarene University
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Barack Wanjawa, Lawrence Muchemi (University of Nairobi), Lilian D.A. Wanzare, Florence Indede, Owen McOnyango (Maseno University), Edward Ombui (Africa Nazarene University)</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ui_62</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>MasakhaNER 2.0: Named Entity Recognition datasets for 20 African languages</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>MasakhaNER 2.0 is the largest human-annotated named entity recognition dataset for 20 African languages. Each language has between 4,800 – 11,000 parallel sentences for training and/or evaluation. The languages covered span across West, Central, East and Southern Africa.</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://github.com/masakhane-io/masakhane-ner/tree/main/MasakhaNER2.0/data</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>David Ifeoluwa Adelani, D.ADELANI@UCL.AC.UK</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Africa (Multi-country)</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Powered by: Multiple collaborating institutions
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>David Ifeoluwa Adelani, Multiple collaborators (Multiple collaborating institutions)</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ui_63</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>MAFAND-MT: Masakhane Anglo &amp; Franco African News Corpus for Machine Translation</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>The MAFAND-MT dataset is a few thousand high-quality and human translated parallel sentences for 16 African languages in the news domain. Each language has between 1,466 – 7838 parallel sentences for training and/or evaluation.</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://github.com/masakhane-io/lafand-mt</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>David Ifeoluwa Adelani, D.ADELANI@UCL.AC.UK</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Africa (Multi-country)</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>Powered by: Multiple collaborating institutions
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>David Ifeoluwa Adelani, Multiple collaborators (Multiple collaborating institutions)</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr"/>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ui_64</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>MasakhaPOS: Part-of-Speech Tagging Dataset for 20 African Languages</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>MasakhaPOS is the largest human-annotated part of speech tagging dataset for 20 African languages. Each language has between 1200 – 1500 sentences for training and/or evaluation. The languages covered span across West, Central, East and Southern Africa.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://github.com/masakhane-io/masakhane-pos</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>David Ifeoluwa Adelani, D.ADELANI@UCL.AC.UK</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Africa (Multi-country)</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Powered by: Multiple collaborating institutions
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>David Ifeoluwa Adelani, Multiple collaborators (Multiple collaborating institutions)</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr"/>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr"/>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ui_65</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Financial Inclusion Speech Dataset for some Ghanaian Languages</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>This speech dataset for the Ghanian languages Akan (Akuapem Twi, Asante Twi, Fante) and Ga includes 104,000 utterances (speech) across the four dialects/languages with approximately 200 speakers per dialect/language. This amounts to about 148 hours of speech in total.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://github.com/Ashesi-Org/Financial-Inclusion-Speech-Dataset</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Dennis Asamoah Owusu, DOWUSU@ASHESI.EDU.GH</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Powered by: Ashesi University and collaborating institutions
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Dennis Asamoah Owusu, Multiple collaborators (Ashesi University and collaborating institutions)</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr"/>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr"/>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ui_66</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>IgboSynCorp: Dataset for Igbo Natural Language Processing Tasks</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>This dataset is the first spoken corpus of labelled and unlabeled datasets for Igbo Natural Language Processing (NLP) tasks. It consists of approximately 40 hours of naturally occurring Igbo speech that is representative of all the dialects of Igbo.</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://dataverse.harvard.edu/dataverse/0000-0002-0068-6933</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Gerald Nweya (GERALDNWEYA@GMAIL.COM) and Emeka Onwuegbuzia (EONWUEGBUZIA@GMAIL.COM)</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Powered by: Igbo NLP research collaboration
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Gerald Nweya, Emeka Onwuegbuzia (Igbo NLP research collaboration)</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr"/>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ui_67</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Bayelemabaga Aligned Bambara-French Corpus for Machine Translation</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>The Bayelemabaga dataset consists of 46,976 parallel machine translation-ready Bambara-French sentence pairs, originating from the Bambara Reference Corpus from INALCO's LLACAN Lab. The text is extracted from 264 text files.</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://robotsmali-ai.github.io/datasets/</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Christopher Homan, christopher.m.homan.phd@gmail.com</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Mali/France</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>Powered by: Multi-institutional collaboration
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Allahsera Auguste Tapo, Michael Leventhal, Valentin Vydrin, Sebastian Diarra, Marcos Zampieri, Emily Prud'Hommeaux, Jean Jacque Méric, Christopher Homan (Multi-institutional collaboration)</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr"/>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ui_68</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Makerere University NLP Datasets</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Makerere University has created text and speech datasets for low-resourced East African Languages in Uganda, Tanzania, and Kenya. This dataset contains 10,000 parallel sentiment-tagged sentences, 100,000 Kiswahili sentences, 100,000 Luganda sentences, 40,037 Acoli sentences, and 39,999 Lumasaaba sentences.</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://dataverse.harvard.edu/dataverse/makerereuniversitylacuna</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Andrew Katumba | andrew.katumba@mak.ac.ug</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Uganda, Tanzania, Kenya</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>Powered by: Makerere University, Maseno University, TYD Innovation Incubator
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Katumba Andrew, Nakatumba-Nabende Joyce, Babirye Claire, Mukiibi Jonathan, Tusubira Jeremy, Bateesa Tobias, Wairagala Eric Peter, Fridah Katushemererwe, Mutebi Chodrine, Nabende Peter, Sentanda Medadi, Ssenkungu Ivan (Makerere University), Wanzare Lilian (Maseno University), Davis David (TYD Innovation Incubator)</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr"/>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr"/>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ui_69</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>BIG-C: A Multimodal Multi-Purpose Dataset for Bemba</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>The BIG-C (Bemba Image Grounded Conversations) dataset is comprised of multi-turn dialogues between Bemba speakers grounded on images, transcribed and translated to English. There are over 92,000 sentences, amounting to over 180 hours of speech data with corresponding Bemba transcriptions and English translations.</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://github.com/csikasote/bigc</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Claytone Sikasote | claytonsikasote@gmail.com</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Zambia</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Powered by: University of Zambia, George Mason University
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Claytone Sikasote, Eunice Mukonde – Mulenga (University of Zambia), Md Mahfuz Ibn Alam, Antonios Anastasopoulos (George Mason University)</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr"/>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ui_70</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>KALLAAMA</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>This dataset will strengthen natural language processing resources for Wolof, Pulaar, and Serer, the three most widely spoken languages in Senegal. This dataset's repository of transcribed speech includes over 55 hours in Wolof, 38 hours in Serer, and 31 hours in Pulaar.</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://github.com/gauthelo/kallaama-speech-dataset</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Aminata Ndiaye | amina.ndiaye@jokalante.com and Elodie Gauthier | elodie.gauthier@orange.com</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Powered by: Jokalante, Dakar, Senegal, Orange Innovation, Lannion, France, Ecole Polytechnique de Thiès, Senegal
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Aminata Ndiaye Diallo (Jokalante, Dakar, Senegal), Elodie Gauthier (Orange Innovation, Lannion, France), Abdoulaye Guissé (Ecole Polytechnique de Thiès, Senegal)</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr"/>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ui_71</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>NaijaVoices: Our Language is Our Strength</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>The NaijaVoices project has curated 1,867 hours of speech and text data featuring over 5,000 speakers in the three major Nigerian languages — Hausa, Igbo, and Yoruba. As of its release, it is the largest ever multi-speaker African speech dataset. The dataset consists of circa 1,917,686 instances.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Not specified in source</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Language Technology</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Language Data</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>info@naijavoices.com</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Powered by: NaijaVoices project
+Catalyzed by: Lacuna-Fund / Meridian (Language-call) &amp; FAIR Forward - AI for All
+Financed by: BMZ</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Multiple contributors (NaijaVoices project)</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>language-banner</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr"/>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>Added via language dataset integration - extracted from language.html</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>